<commit_message>
feat(equity-valuation): surface analysis in app + add analyze.bat launcher
- app.py now shows the financial-statement & quality analysis (F-Score, Altman Z,
  Beneish M, Sloan, ROIC vs WACC, reverse DCF) under the valuation, with the full note
- analyze.bat: double-click launcher for the research workup
</commit_message>
<xml_diff>
--- a/equity-valuation/output/NVDA_valuation.xlsx
+++ b/equity-valuation/output/NVDA_valuation.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0)"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,9 +45,6 @@
     </font>
     <font>
       <color rgb="000F172A"/>
-    </font>
-    <font>
-      <color rgb="001D4ED8"/>
     </font>
     <font>
       <b val="1"/>
@@ -88,25 +85,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,7 +492,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Blue = input (editable). Fundamentals from SEC EDGAR; market/assumptions flagged.</t>
+          <t>Editable inputs on this tab. Fundamentals from SEC EDGAR; market/assumptions flagged.</t>
         </is>
       </c>
     </row>
@@ -845,23 +838,23 @@
       <c r="E4" s="7" t="n">
         <v>215938</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="7">
         <f>E4*(1+Assumptions!B19)</f>
         <v/>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="7">
         <f>F4*(1+Assumptions!B20)</f>
         <v/>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="7">
         <f>G4*(1+Assumptions!B21)</f>
         <v/>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="7">
         <f>H4*(1+Assumptions!B22)</f>
         <v/>
       </c>
-      <c r="J4" s="10">
+      <c r="J4" s="7">
         <f>I4*(1+Assumptions!B23)</f>
         <v/>
       </c>
@@ -884,23 +877,23 @@
       <c r="E5" s="7" t="n">
         <v>130387</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="7">
         <f>F4*Assumptions!B26</f>
         <v/>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="7">
         <f>G4*Assumptions!B27</f>
         <v/>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="7">
         <f>H4*Assumptions!B28</f>
         <v/>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="7">
         <f>I4*Assumptions!B29</f>
         <v/>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="7">
         <f>J4*Assumptions!B30</f>
         <v/>
       </c>
@@ -911,39 +904,39 @@
           <t>EBIT margin (%)</t>
         </is>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="4">
         <f>B5/B4</f>
         <v/>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="4">
         <f>C5/C4</f>
         <v/>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="4">
         <f>D5/D4</f>
         <v/>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="4">
         <f>E5/E4</f>
         <v/>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="4">
         <f>F5/F4</f>
         <v/>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="4">
         <f>G5/G4</f>
         <v/>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="4">
         <f>H5/H4</f>
         <v/>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="4">
         <f>I5/I4</f>
         <v/>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="4">
         <f>J5/J4</f>
         <v/>
       </c>
@@ -999,23 +992,23 @@
           <t>NOPAT ($m)</t>
         </is>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="7">
         <f>F5*(1-Assumptions!B4)</f>
         <v/>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="7">
         <f>G5*(1-Assumptions!B4)</f>
         <v/>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="7">
         <f>H5*(1-Assumptions!B4)</f>
         <v/>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="7">
         <f>I5*(1-Assumptions!B4)</f>
         <v/>
       </c>
-      <c r="J11" s="10">
+      <c r="J11" s="7">
         <f>J5*(1-Assumptions!B4)</f>
         <v/>
       </c>
@@ -1026,23 +1019,23 @@
           <t>D&amp;A ($m)</t>
         </is>
       </c>
-      <c r="F12" s="10">
+      <c r="F12" s="7">
         <f>F4*Assumptions!B12</f>
         <v/>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="7">
         <f>G4*Assumptions!B12</f>
         <v/>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="7">
         <f>H4*Assumptions!B12</f>
         <v/>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="7">
         <f>I4*Assumptions!B12</f>
         <v/>
       </c>
-      <c r="J12" s="10">
+      <c r="J12" s="7">
         <f>J4*Assumptions!B12</f>
         <v/>
       </c>
@@ -1053,23 +1046,23 @@
           <t>Capex ($m)</t>
         </is>
       </c>
-      <c r="F13" s="10">
+      <c r="F13" s="7">
         <f>F4*Assumptions!B13</f>
         <v/>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="7">
         <f>G4*Assumptions!B13</f>
         <v/>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="7">
         <f>H4*Assumptions!B13</f>
         <v/>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="7">
         <f>I4*Assumptions!B13</f>
         <v/>
       </c>
-      <c r="J13" s="10">
+      <c r="J13" s="7">
         <f>J4*Assumptions!B13</f>
         <v/>
       </c>
@@ -1080,23 +1073,23 @@
           <t>Incr. NWC ($m)</t>
         </is>
       </c>
-      <c r="F14" s="10">
+      <c r="F14" s="7">
         <f>(F4-E4)*Assumptions!B14</f>
         <v/>
       </c>
-      <c r="G14" s="10">
+      <c r="G14" s="7">
         <f>(G4-F4)*Assumptions!B14</f>
         <v/>
       </c>
-      <c r="H14" s="10">
+      <c r="H14" s="7">
         <f>(H4-G4)*Assumptions!B14</f>
         <v/>
       </c>
-      <c r="I14" s="10">
+      <c r="I14" s="7">
         <f>(I4-H4)*Assumptions!B14</f>
         <v/>
       </c>
-      <c r="J14" s="10">
+      <c r="J14" s="7">
         <f>(J4-I4)*Assumptions!B14</f>
         <v/>
       </c>
@@ -1107,23 +1100,23 @@
           <t>FCFF ($m)</t>
         </is>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="7">
         <f>F11+F12-F13-F14</f>
         <v/>
       </c>
-      <c r="G15" s="10">
+      <c r="G15" s="7">
         <f>G11+G12-G13-G14</f>
         <v/>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="7">
         <f>H11+H12-H13-H14</f>
         <v/>
       </c>
-      <c r="I15" s="10">
+      <c r="I15" s="7">
         <f>I11+I12-I13-I14</f>
         <v/>
       </c>
-      <c r="J15" s="10">
+      <c r="J15" s="7">
         <f>J11+J12-J13-J14</f>
         <v/>
       </c>
@@ -1159,7 +1152,7 @@
           <t>Cost of equity (CAPM)</t>
         </is>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="4">
         <f>Assumptions!B5+Assumptions!B7*Assumptions!B6</f>
         <v/>
       </c>
@@ -1170,7 +1163,7 @@
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="4">
         <f>Assumptions!B8*(1-Assumptions!B4)</f>
         <v/>
       </c>
@@ -1181,7 +1174,7 @@
           <t>Equity value ($m)</t>
         </is>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="7">
         <f>Assumptions!B9*Assumptions!B10</f>
         <v/>
       </c>
@@ -1192,7 +1185,7 @@
           <t>Debt value ($m)</t>
         </is>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="7">
         <f>Assumptions!B15</f>
         <v/>
       </c>
@@ -1203,7 +1196,7 @@
           <t>Equity weight</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="4">
         <f>B6/(B6+B7)</f>
         <v/>
       </c>
@@ -1214,7 +1207,7 @@
           <t>Debt weight</t>
         </is>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="4">
         <f>B7/(B6+B7)</f>
         <v/>
       </c>
@@ -1225,7 +1218,7 @@
           <t>WACC</t>
         </is>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="10">
         <f>B8*B4+B9*B5</f>
         <v/>
       </c>
@@ -1287,23 +1280,23 @@
           <t>FCFF ($m)</t>
         </is>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="7">
         <f>Model!F15</f>
         <v/>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="7">
         <f>Model!G15</f>
         <v/>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="7">
         <f>Model!H15</f>
         <v/>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="7">
         <f>Model!I15</f>
         <v/>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="7">
         <f>Model!J15</f>
         <v/>
       </c>
@@ -1314,23 +1307,23 @@
           <t>Discount factor</t>
         </is>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="5">
         <f>1/(1+WACC!$B$10)^B3</f>
         <v/>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="5">
         <f>1/(1+WACC!$B$10)^C3</f>
         <v/>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="5">
         <f>1/(1+WACC!$B$10)^D3</f>
         <v/>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="5">
         <f>1/(1+WACC!$B$10)^E3</f>
         <v/>
       </c>
-      <c r="F5" s="13">
+      <c r="F5" s="5">
         <f>1/(1+WACC!$B$10)^F3</f>
         <v/>
       </c>
@@ -1341,23 +1334,23 @@
           <t>PV of FCFF ($m)</t>
         </is>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="7">
         <f>B4*B5</f>
         <v/>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="7">
         <f>C4*C5</f>
         <v/>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="7">
         <f>D4*D5</f>
         <v/>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="7">
         <f>E4*E5</f>
         <v/>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="7">
         <f>F4*F5</f>
         <v/>
       </c>
@@ -1368,7 +1361,7 @@
           <t>Sum PV of FCFF ($m)</t>
         </is>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="7">
         <f>SUM(B6:F6)</f>
         <v/>
       </c>
@@ -1379,7 +1372,7 @@
           <t>Terminal value ($m)</t>
         </is>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="7">
         <f>F4*(1+Assumptions!B11)/(WACC!B10-Assumptions!B11)</f>
         <v/>
       </c>
@@ -1390,7 +1383,7 @@
           <t>PV of terminal value ($m)</t>
         </is>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="7">
         <f>B9*F5</f>
         <v/>
       </c>
@@ -1401,7 +1394,7 @@
           <t>Enterprise value ($m)</t>
         </is>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="7">
         <f>B8+B10</f>
         <v/>
       </c>
@@ -1412,7 +1405,7 @@
           <t>Less: net debt ($m)</t>
         </is>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="7">
         <f>Assumptions!B15-Assumptions!B16</f>
         <v/>
       </c>
@@ -1423,7 +1416,7 @@
           <t>Equity value ($m)</t>
         </is>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="7">
         <f>B11-B12</f>
         <v/>
       </c>
@@ -1434,7 +1427,7 @@
           <t>Shares (m)</t>
         </is>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="7">
         <f>Assumptions!B10</f>
         <v/>
       </c>
@@ -1445,7 +1438,7 @@
           <t>Value per share ($)</t>
         </is>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="11">
         <f>B13/B14</f>
         <v/>
       </c>
@@ -1456,7 +1449,7 @@
           <t>TV as % of EV</t>
         </is>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="4">
         <f>B10/B11</f>
         <v/>
       </c>
@@ -1514,131 +1507,131 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="11">
+      <c r="B4" s="4">
         <f>WACC!$B$10-0.015</f>
         <v/>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B4)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+C$3)/($B4-C$3))/(1+$B4)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="D4" s="15">
+      <c r="D4" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B4)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+D$3)/($B4-D$3))/(1+$B4)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B4)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+E$3)/($B4-E$3))/(1+$B4)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="F4" s="15">
+      <c r="F4" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B4)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+F$3)/($B4-F$3))/(1+$B4)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="G4" s="15">
+      <c r="G4" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B4)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+G$3)/($B4-G$3))/(1+$B4)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="11">
+      <c r="B5" s="4">
         <f>WACC!$B$10-0.0075</f>
         <v/>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B5)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+C$3)/($B5-C$3))/(1+$B5)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B5)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+D$3)/($B5-D$3))/(1+$B5)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B5)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+E$3)/($B5-E$3))/(1+$B5)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B5)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+F$3)/($B5-F$3))/(1+$B5)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B5)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+G$3)/($B5-G$3))/(1+$B5)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="11">
+      <c r="B6" s="4">
         <f>WACC!$B$10</f>
         <v/>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B6)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+C$3)/($B6-C$3))/(1+$B6)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B6)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+D$3)/($B6-D$3))/(1+$B6)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="11">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B6)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+E$3)/($B6-E$3))/(1+$B6)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B6)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+F$3)/($B6-F$3))/(1+$B6)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B6)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+G$3)/($B6-G$3))/(1+$B6)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="11">
+      <c r="B7" s="4">
         <f>WACC!$B$10+0.0075</f>
         <v/>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B7)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+C$3)/($B7-C$3))/(1+$B7)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B7)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+D$3)/($B7-D$3))/(1+$B7)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B7)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+E$3)/($B7-E$3))/(1+$B7)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B7)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+F$3)/($B7-F$3))/(1+$B7)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B7)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+G$3)/($B7-G$3))/(1+$B7)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="11">
+      <c r="B8" s="4">
         <f>WACC!$B$10+0.015</f>
         <v/>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B8)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+C$3)/($B8-C$3))/(1+$B8)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B8)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+D$3)/($B8-D$3))/(1+$B8)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B8)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+E$3)/($B8-E$3))/(1+$B8)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B8)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+F$3)/($B8-F$3))/(1+$B8)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="6">
         <f>(SUMPRODUCT(DCF!$B$4:$F$4,1/(1+$B8)^DCF!$B$3:$F$3)+(DCF!$F$4*(1+G$3)/($B8-G$3))/(1+$B8)^5-(Assumptions!B15-Assumptions!B16))/Assumptions!B10</f>
         <v/>
       </c>
@@ -1701,7 +1694,7 @@
           <t>Implied EV ($m)</t>
         </is>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="7">
         <f>B4*B5</f>
         <v/>
       </c>
@@ -1712,7 +1705,7 @@
           <t>Less: net debt ($m)</t>
         </is>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="7">
         <f>Assumptions!B15-Assumptions!B16</f>
         <v/>
       </c>
@@ -1723,7 +1716,7 @@
           <t>Equity value ($m)</t>
         </is>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="7">
         <f>B6-B7</f>
         <v/>
       </c>
@@ -1734,7 +1727,7 @@
           <t>Value/share — EV/EBITDA ($)</t>
         </is>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="6">
         <f>B8/Assumptions!B10</f>
         <v/>
       </c>
@@ -1765,7 +1758,7 @@
           <t>Value/share — P/E ($)</t>
         </is>
       </c>
-      <c r="B13" s="15">
+      <c r="B13" s="6">
         <f>B11*B12</f>
         <v/>
       </c>
@@ -1776,7 +1769,7 @@
           <t>Comps midpoint ($)</t>
         </is>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="11">
         <f>AVERAGE(B9,B13)</f>
         <v/>
       </c>

</xml_diff>